<commit_message>
Update logic in caculation
</commit_message>
<xml_diff>
--- a/data/Apr/InternalDailyReport_Apr.xlsx
+++ b/data/Apr/InternalDailyReport_Apr.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Work\Freelance\TextInputter\data\Apr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3861460-BDC1-42A2-B9E5-B0634DFB6C4C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E18E296-7ED7-47D4-96AA-558D25F193B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="11" activeTab="20" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="1000" activeTab="25" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="01-04" sheetId="2" r:id="rId1"/>
@@ -10069,11 +10069,11 @@
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="3" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="3" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
@@ -11374,11 +11374,11 @@
       <c r="B28" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C28" s="49">
+      <c r="C28" s="48">
         <f>SUMIFS(I$3:I$23,B$3:B$23,A$27,L$3:L$23,A$28)</f>
         <v>11295</v>
       </c>
-      <c r="D28" s="49"/>
+      <c r="D28" s="48"/>
       <c r="E28" s="3">
         <f>SUMIFS(Q$3:Q$23,B$3:B$23,A$27,L$3:L$23,A$28)</f>
         <v>21</v>
@@ -11409,10 +11409,10 @@
       <c r="B29" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C29" s="46">
+      <c r="C29" s="49">
         <v>0</v>
       </c>
-      <c r="D29" s="46"/>
+      <c r="D29" s="49"/>
       <c r="K29" t="s">
         <v>98</v>
       </c>
@@ -11436,11 +11436,11 @@
       <c r="B30" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C30" s="46">
+      <c r="C30" s="49">
         <f>-SUMIFS(I$3:I$23,B$3:B$23,A$27,P$3:P$23,"xx",N$3:N$23,"x")</f>
         <v>0</v>
       </c>
-      <c r="D30" s="46"/>
+      <c r="D30" s="49"/>
       <c r="E30" s="2">
         <f>SUMIFS(Q$3:Q$23,B$3:B$23,A$27,P$3:P$23,"xx",N$3:N$23,"x")</f>
         <v>0</v>
@@ -11484,8 +11484,8 @@
       <c r="B32" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C32" s="48"/>
-      <c r="D32" s="48"/>
+      <c r="C32" s="45"/>
+      <c r="D32" s="45"/>
       <c r="K32" s="2" t="s">
         <v>105</v>
       </c>
@@ -11501,8 +11501,8 @@
       <c r="B33" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C33" s="48"/>
-      <c r="D33" s="48"/>
+      <c r="C33" s="45"/>
+      <c r="D33" s="45"/>
       <c r="L33" s="9">
         <f>SUBTOTAL(9,L28:L32)</f>
         <v>7314</v>
@@ -11516,11 +11516,11 @@
       <c r="B35" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C35" s="45">
+      <c r="C35" s="46">
         <f>C31+C32+C33</f>
         <v>11295</v>
       </c>
-      <c r="D35" s="45"/>
+      <c r="D35" s="46"/>
       <c r="E35" s="1" t="s">
         <v>109</v>
       </c>
@@ -13652,11 +13652,11 @@
       <c r="B48" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C48" s="49">
+      <c r="C48" s="48">
         <f>SUMIFS(I$3:I$43,B$3:B$43,A$47,L$3:L$43,A$48)</f>
         <v>28800</v>
       </c>
-      <c r="D48" s="49"/>
+      <c r="D48" s="48"/>
       <c r="E48" s="3">
         <f>SUMIFS(Q$3:Q$43,B$3:B$43,A$47,L$3:L$43,A$48)</f>
         <v>41</v>
@@ -13691,10 +13691,10 @@
       <c r="B49" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C49" s="46">
+      <c r="C49" s="49">
         <v>0</v>
       </c>
-      <c r="D49" s="46"/>
+      <c r="D49" s="49"/>
       <c r="K49" t="s">
         <v>98</v>
       </c>
@@ -13718,11 +13718,11 @@
       <c r="B50" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C50" s="46">
+      <c r="C50" s="49">
         <f>-SUMIFS(I$3:I$43,B$3:B$43,A$47,P$3:P$43,"xx",N$3:N$43,"x")</f>
         <v>0</v>
       </c>
-      <c r="D50" s="46"/>
+      <c r="D50" s="49"/>
       <c r="E50" s="2">
         <f>SUMIFS(Q$3:Q$43,B$3:B$43,A$47,P$3:P$43,"xx",N$3:N$43,"x")</f>
         <v>0</v>
@@ -13774,8 +13774,8 @@
       <c r="B52" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C52" s="48"/>
-      <c r="D52" s="48"/>
+      <c r="C52" s="45"/>
+      <c r="D52" s="45"/>
       <c r="K52" s="2" t="s">
         <v>105</v>
       </c>
@@ -13791,8 +13791,8 @@
       <c r="B53" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C53" s="48"/>
-      <c r="D53" s="48"/>
+      <c r="C53" s="45"/>
+      <c r="D53" s="45"/>
       <c r="L53" s="9">
         <f>SUBTOTAL(9,L48:L52)</f>
         <v>3498</v>
@@ -13813,11 +13813,11 @@
       <c r="B55" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C55" s="45">
+      <c r="C55" s="46">
         <f>C51+C52+C53</f>
         <v>28800</v>
       </c>
-      <c r="D55" s="45"/>
+      <c r="D55" s="46"/>
       <c r="E55" s="1" t="s">
         <v>109</v>
       </c>
@@ -17033,11 +17033,11 @@
       <c r="B71" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C71" s="49">
+      <c r="C71" s="48">
         <f>SUMIFS(I$3:I$66,B$3:B$66,A$70,L$3:L$66,A$71)</f>
         <v>40275</v>
       </c>
-      <c r="D71" s="49"/>
+      <c r="D71" s="48"/>
       <c r="E71" s="3">
         <f>SUMIFS(Q$3:Q$66,B$3:B$66,A$70,L$3:L$66,A$71)</f>
         <v>63</v>
@@ -17072,10 +17072,10 @@
       <c r="B72" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C72" s="46">
+      <c r="C72" s="49">
         <v>0</v>
       </c>
-      <c r="D72" s="46"/>
+      <c r="D72" s="49"/>
       <c r="K72" t="s">
         <v>98</v>
       </c>
@@ -17099,11 +17099,11 @@
       <c r="B73" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C73" s="46">
+      <c r="C73" s="49">
         <f>-SUMIFS(I$3:I$66,B$3:B$66,A$70,P$3:P$66,"xx",N$3:N$66,"x")</f>
         <v>-790</v>
       </c>
-      <c r="D73" s="46"/>
+      <c r="D73" s="49"/>
       <c r="E73" s="2">
         <f>SUMIFS(Q$3:Q$66,B$3:B$66,A$70,P$3:P$66,"xx",N$3:N$66,"x")</f>
         <v>1</v>
@@ -17147,8 +17147,8 @@
       <c r="B75" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C75" s="48"/>
-      <c r="D75" s="48"/>
+      <c r="C75" s="45"/>
+      <c r="D75" s="45"/>
       <c r="K75" s="2" t="s">
         <v>105</v>
       </c>
@@ -17164,8 +17164,8 @@
       <c r="B76" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C76" s="48"/>
-      <c r="D76" s="48"/>
+      <c r="C76" s="45"/>
+      <c r="D76" s="45"/>
       <c r="L76" s="9">
         <f>SUBTOTAL(9,L71:L75)</f>
         <v>15833</v>
@@ -17194,11 +17194,11 @@
       <c r="B78" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C78" s="45">
+      <c r="C78" s="46">
         <f>C74+C75+C76</f>
         <v>39485</v>
       </c>
-      <c r="D78" s="45"/>
+      <c r="D78" s="46"/>
       <c r="E78" s="1" t="s">
         <v>109</v>
       </c>
@@ -18681,11 +18681,11 @@
       <c r="B31" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C31" s="49">
+      <c r="C31" s="48">
         <f>SUMIFS(I$3:I$26,B$3:B$26,A$30,L$3:L$26,A$31)</f>
         <v>10860</v>
       </c>
-      <c r="D31" s="49"/>
+      <c r="D31" s="48"/>
       <c r="E31" s="3">
         <f>SUMIFS(Q$3:Q$26,B$3:B$26,A$30,L$3:L$26,A$31)</f>
         <v>20</v>
@@ -18720,10 +18720,10 @@
       <c r="B32" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C32" s="46">
+      <c r="C32" s="49">
         <v>0</v>
       </c>
-      <c r="D32" s="46"/>
+      <c r="D32" s="49"/>
       <c r="K32" t="s">
         <v>98</v>
       </c>
@@ -18747,11 +18747,11 @@
       <c r="B33" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C33" s="46">
+      <c r="C33" s="49">
         <f>-SUMIFS(I$3:I$26,B$3:B$26,A$30,P$3:P$26,"xx",N$3:N$26,"x")</f>
         <v>-2910</v>
       </c>
-      <c r="D33" s="46"/>
+      <c r="D33" s="49"/>
       <c r="E33" s="2">
         <f>SUMIFS(Q$3:Q$26,B$3:B$26,A$30,P$3:P$26,"xx",N$3:N$26,"x")</f>
         <v>4</v>
@@ -18801,8 +18801,8 @@
       <c r="B35" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C35" s="48"/>
-      <c r="D35" s="48"/>
+      <c r="C35" s="45"/>
+      <c r="D35" s="45"/>
       <c r="K35" s="2" t="s">
         <v>105</v>
       </c>
@@ -18818,8 +18818,8 @@
       <c r="B36" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C36" s="48"/>
-      <c r="D36" s="48"/>
+      <c r="C36" s="45"/>
+      <c r="D36" s="45"/>
       <c r="L36" s="9">
         <f>SUBTOTAL(9,L31:L35)</f>
         <v>-328</v>
@@ -18840,11 +18840,11 @@
       <c r="B38" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C38" s="45">
+      <c r="C38" s="46">
         <f>C34+C35+C36</f>
         <v>7950</v>
       </c>
-      <c r="D38" s="45"/>
+      <c r="D38" s="46"/>
       <c r="E38" s="1" t="s">
         <v>109</v>
       </c>
@@ -20686,11 +20686,11 @@
       <c r="B40" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C40" s="49">
+      <c r="C40" s="48">
         <f>SUMIFS(I$3:I$35,B$3:B$35,A$39,L$3:L$35,A$40)</f>
         <v>22860</v>
       </c>
-      <c r="D40" s="49"/>
+      <c r="D40" s="48"/>
       <c r="E40" s="3">
         <f>SUMIFS(Q$3:Q$35,B$3:B$35,A$39,L$3:L$35,A$40)</f>
         <v>32</v>
@@ -20725,10 +20725,10 @@
       <c r="B41" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C41" s="46">
+      <c r="C41" s="49">
         <v>0</v>
       </c>
-      <c r="D41" s="46"/>
+      <c r="D41" s="49"/>
       <c r="K41" t="s">
         <v>98</v>
       </c>
@@ -20752,11 +20752,11 @@
       <c r="B42" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C42" s="46">
+      <c r="C42" s="49">
         <f>-SUMIFS(I$3:I$35,B$3:B$35,A$39,P$3:P$35,"xx",N$3:N$35,"x")</f>
         <v>-870</v>
       </c>
-      <c r="D42" s="46"/>
+      <c r="D42" s="49"/>
       <c r="E42" s="2">
         <f>SUMIFS(Q$3:Q$35,B$3:B$35,A$39,P$3:P$35,"xx",N$3:N$35,"x")</f>
         <v>1</v>
@@ -20800,8 +20800,8 @@
       <c r="B44" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C44" s="48"/>
-      <c r="D44" s="48"/>
+      <c r="C44" s="45"/>
+      <c r="D44" s="45"/>
       <c r="K44" s="2" t="s">
         <v>105</v>
       </c>
@@ -20817,8 +20817,8 @@
       <c r="B45" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C45" s="48"/>
-      <c r="D45" s="48"/>
+      <c r="C45" s="45"/>
+      <c r="D45" s="45"/>
       <c r="L45" s="9">
         <f>SUBTOTAL(9,L40:L44)</f>
         <v>5050</v>
@@ -20839,11 +20839,11 @@
       <c r="B47" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C47" s="45">
+      <c r="C47" s="46">
         <f>C43+C44+C45</f>
         <v>21990</v>
       </c>
-      <c r="D47" s="45"/>
+      <c r="D47" s="46"/>
       <c r="E47" s="1" t="s">
         <v>109</v>
       </c>
@@ -23450,11 +23450,11 @@
       <c r="B57" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C57" s="49">
+      <c r="C57" s="48">
         <f>SUMIFS(I$3:I$52,B$3:B$52,A$56,L$3:L$52,A$57)</f>
         <v>28155</v>
       </c>
-      <c r="D57" s="49"/>
+      <c r="D57" s="48"/>
       <c r="E57" s="3">
         <f>SUMIFS(Q$3:Q$52,B$3:B$52,A$56,L$3:L$52,A$57)</f>
         <v>49</v>
@@ -23485,10 +23485,10 @@
       <c r="B58" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C58" s="46">
+      <c r="C58" s="49">
         <v>0</v>
       </c>
-      <c r="D58" s="46"/>
+      <c r="D58" s="49"/>
       <c r="K58" t="s">
         <v>98</v>
       </c>
@@ -23512,11 +23512,11 @@
       <c r="B59" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C59" s="46">
+      <c r="C59" s="49">
         <f>-SUMIFS(I$3:I$52,B$3:B$52,A$56,P$3:P$52,"xx",N$3:N$52,"x")</f>
         <v>-3155</v>
       </c>
-      <c r="D59" s="46"/>
+      <c r="D59" s="49"/>
       <c r="E59" s="2">
         <f>SUMIFS(Q$3:Q$52,B$3:B$52,A$56,P$3:P$52,"xx",N$3:N$52,"x")</f>
         <v>2</v>
@@ -23560,8 +23560,8 @@
       <c r="B61" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C61" s="48"/>
-      <c r="D61" s="48"/>
+      <c r="C61" s="45"/>
+      <c r="D61" s="45"/>
       <c r="K61" s="2" t="s">
         <v>105</v>
       </c>
@@ -23577,8 +23577,8 @@
       <c r="B62" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C62" s="48"/>
-      <c r="D62" s="48"/>
+      <c r="C62" s="45"/>
+      <c r="D62" s="45"/>
       <c r="L62" s="9">
         <f>SUBTOTAL(9,L57:L61)</f>
         <v>7146</v>
@@ -23599,11 +23599,11 @@
       <c r="B64" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C64" s="45">
+      <c r="C64" s="46">
         <f>C60+C61+C62</f>
         <v>25000</v>
       </c>
-      <c r="D64" s="45"/>
+      <c r="D64" s="46"/>
       <c r="E64" s="1" t="s">
         <v>109</v>
       </c>
@@ -26243,11 +26243,11 @@
       <c r="B58" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C58" s="49">
+      <c r="C58" s="48">
         <f>SUMIFS(I$3:I$53,B$3:B$53,A$57,L$3:L$53,A$58)</f>
         <v>30480</v>
       </c>
-      <c r="D58" s="49"/>
+      <c r="D58" s="48"/>
       <c r="E58" s="3">
         <f>SUMIFS(Q$3:Q$53,B$3:B$53,A$57,L$3:L$53,A$58)</f>
         <v>51</v>
@@ -26282,10 +26282,10 @@
       <c r="B59" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C59" s="46">
+      <c r="C59" s="49">
         <v>0</v>
       </c>
-      <c r="D59" s="46"/>
+      <c r="D59" s="49"/>
       <c r="K59" t="s">
         <v>98</v>
       </c>
@@ -26309,11 +26309,11 @@
       <c r="B60" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C60" s="46">
+      <c r="C60" s="49">
         <f>-SUMIFS(I$3:I$53,B$3:B$53,A$57,P$3:P$53,"xx",N$3:N$53,"x")</f>
         <v>0</v>
       </c>
-      <c r="D60" s="46"/>
+      <c r="D60" s="49"/>
       <c r="E60" s="2">
         <f>SUMIFS(Q$3:Q$53,B$3:B$53,A$57,P$3:P$53,"xx",N$3:N$53,"x")</f>
         <v>0</v>
@@ -26357,8 +26357,8 @@
       <c r="B62" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C62" s="48"/>
-      <c r="D62" s="48"/>
+      <c r="C62" s="45"/>
+      <c r="D62" s="45"/>
       <c r="K62" s="2" t="s">
         <v>105</v>
       </c>
@@ -26374,8 +26374,8 @@
       <c r="B63" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C63" s="48"/>
-      <c r="D63" s="48"/>
+      <c r="C63" s="45"/>
+      <c r="D63" s="45"/>
       <c r="L63" s="9">
         <f>SUBTOTAL(9,L58:L62)</f>
         <v>13705</v>
@@ -26396,11 +26396,11 @@
       <c r="B65" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C65" s="45">
+      <c r="C65" s="46">
         <f>C61+C62+C63</f>
         <v>30480</v>
       </c>
-      <c r="D65" s="45"/>
+      <c r="D65" s="46"/>
       <c r="E65" s="1" t="s">
         <v>109</v>
       </c>
@@ -28399,11 +28399,11 @@
       <c r="B43" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C43" s="49">
+      <c r="C43" s="48">
         <f>SUMIFS(I$3:I$38,B$3:B$38,A$42,L$3:L$38,A$43)</f>
         <v>16055</v>
       </c>
-      <c r="D43" s="49"/>
+      <c r="D43" s="48"/>
       <c r="E43" s="3">
         <f>SUMIFS(Q$3:Q$38,B$3:B$38,A$42,L$3:L$38,A$43)</f>
         <v>33</v>
@@ -28434,10 +28434,10 @@
       <c r="B44" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C44" s="46">
+      <c r="C44" s="49">
         <v>0</v>
       </c>
-      <c r="D44" s="46"/>
+      <c r="D44" s="49"/>
       <c r="K44" t="s">
         <v>98</v>
       </c>
@@ -28461,11 +28461,11 @@
       <c r="B45" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C45" s="46">
+      <c r="C45" s="49">
         <f>-SUMIFS(I$3:I$38,B$3:B$38,A$42,P$3:P$38,"xx",N$3:N$38,"x")</f>
         <v>-3310</v>
       </c>
-      <c r="D45" s="46"/>
+      <c r="D45" s="49"/>
       <c r="E45" s="2">
         <f>SUMIFS(Q$3:Q$38,B$3:B$38,A$42,P$3:P$38,"xx",N$3:N$38,"x")</f>
         <v>4</v>
@@ -28509,8 +28509,8 @@
       <c r="B47" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C47" s="48"/>
-      <c r="D47" s="48"/>
+      <c r="C47" s="45"/>
+      <c r="D47" s="45"/>
       <c r="K47" s="2" t="s">
         <v>105</v>
       </c>
@@ -28532,8 +28532,8 @@
       <c r="B48" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C48" s="48"/>
-      <c r="D48" s="48"/>
+      <c r="C48" s="45"/>
+      <c r="D48" s="45"/>
       <c r="L48" s="9">
         <f>SUBTOTAL(9,L43:L47)</f>
         <v>840</v>
@@ -28554,11 +28554,11 @@
       <c r="B50" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C50" s="45">
+      <c r="C50" s="46">
         <f>C46+C47+C48</f>
         <v>12745</v>
       </c>
-      <c r="D50" s="45"/>
+      <c r="D50" s="46"/>
       <c r="E50" s="1" t="s">
         <v>109</v>
       </c>
@@ -33164,11 +33164,11 @@
       <c r="B102" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C102" s="49">
+      <c r="C102" s="48">
         <f>SUMIFS(I$3:I$97,B$3:B$97,A$101,L$3:L$97,A$102)</f>
         <v>56435</v>
       </c>
-      <c r="D102" s="49"/>
+      <c r="D102" s="48"/>
       <c r="E102" s="3">
         <f>SUMIFS(Q$3:Q$97,B$3:B$97,A$101,L$3:L$97,A$102)</f>
         <v>95</v>
@@ -33203,10 +33203,10 @@
       <c r="B103" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C103" s="46">
+      <c r="C103" s="49">
         <v>0</v>
       </c>
-      <c r="D103" s="46"/>
+      <c r="D103" s="49"/>
       <c r="K103" t="s">
         <v>98</v>
       </c>
@@ -33230,11 +33230,11 @@
       <c r="B104" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C104" s="46">
+      <c r="C104" s="49">
         <f>-SUMIFS(I$3:I$97,B$3:B$97,A$101,P$3:P$97,"xx",N$3:N$97,"x")</f>
         <v>-2780</v>
       </c>
-      <c r="D104" s="46"/>
+      <c r="D104" s="49"/>
       <c r="E104" s="2">
         <f>SUMIFS(Q$3:Q$97,B$3:B$97,A$101,P$3:P$97,"xx",N$3:N$97,"x")</f>
         <v>3</v>
@@ -33278,8 +33278,8 @@
       <c r="B106" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C106" s="48"/>
-      <c r="D106" s="48"/>
+      <c r="C106" s="45"/>
+      <c r="D106" s="45"/>
       <c r="K106" s="2" t="s">
         <v>105</v>
       </c>
@@ -33295,8 +33295,8 @@
       <c r="B107" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C107" s="48"/>
-      <c r="D107" s="48"/>
+      <c r="C107" s="45"/>
+      <c r="D107" s="45"/>
       <c r="L107" s="9">
         <f>SUBTOTAL(9,L102:L106)</f>
         <v>8245</v>
@@ -33317,11 +33317,11 @@
       <c r="B109" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C109" s="45">
+      <c r="C109" s="46">
         <f>C105+C106+C107</f>
         <v>53655</v>
       </c>
-      <c r="D109" s="45"/>
+      <c r="D109" s="46"/>
       <c r="E109" s="1" t="s">
         <v>109</v>
       </c>
@@ -36481,11 +36481,11 @@
       <c r="B69" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C69" s="49">
+      <c r="C69" s="48">
         <f>SUMIFS(I$3:I$64,B$3:B$64,A$68,L$3:L$64,A$69)</f>
         <v>47670</v>
       </c>
-      <c r="D69" s="49"/>
+      <c r="D69" s="48"/>
       <c r="E69" s="3">
         <f>SUMIFS(Q$3:Q$64,B$3:B$64,A$68,L$3:L$64,A$69)</f>
         <v>58</v>
@@ -36520,10 +36520,10 @@
       <c r="B70" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C70" s="46">
+      <c r="C70" s="49">
         <v>0</v>
       </c>
-      <c r="D70" s="46"/>
+      <c r="D70" s="49"/>
       <c r="K70" t="s">
         <v>98</v>
       </c>
@@ -36547,11 +36547,11 @@
       <c r="B71" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C71" s="46">
+      <c r="C71" s="49">
         <f>-SUMIFS(I$3:I$64,B$3:B$64,A$68,P$3:P$64,"xx",N$3:N$64,"x")</f>
         <v>-5360</v>
       </c>
-      <c r="D71" s="46"/>
+      <c r="D71" s="49"/>
       <c r="E71" s="2">
         <f>SUMIFS(Q$3:Q$64,B$3:B$64,A$68,P$3:P$64,"xx",N$3:N$64,"x")</f>
         <v>5</v>
@@ -36595,8 +36595,8 @@
       <c r="B73" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C73" s="48"/>
-      <c r="D73" s="48"/>
+      <c r="C73" s="45"/>
+      <c r="D73" s="45"/>
       <c r="K73" s="2" t="s">
         <v>105</v>
       </c>
@@ -36612,8 +36612,8 @@
       <c r="B74" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C74" s="48"/>
-      <c r="D74" s="48"/>
+      <c r="C74" s="45"/>
+      <c r="D74" s="45"/>
       <c r="L74" s="9">
         <f>SUBTOTAL(9,L69:L73)</f>
         <v>6850</v>
@@ -36634,11 +36634,11 @@
       <c r="B76" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C76" s="45">
+      <c r="C76" s="46">
         <f>C72+C73+C74</f>
         <v>42310</v>
       </c>
-      <c r="D76" s="45"/>
+      <c r="D76" s="46"/>
       <c r="E76" s="1" t="s">
         <v>109</v>
       </c>
@@ -39422,11 +39422,11 @@
       <c r="B61" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C61" s="49">
+      <c r="C61" s="48">
         <f>SUMIFS(I$3:I$56,B$3:B$56,A$60,L$3:L$56,A$61)</f>
         <v>50515</v>
       </c>
-      <c r="D61" s="49"/>
+      <c r="D61" s="48"/>
       <c r="E61" s="3">
         <f>SUMIFS(Q$3:Q$56,B$3:B$56,A$60,L$3:L$56,A$61)</f>
         <v>54</v>
@@ -39461,10 +39461,10 @@
       <c r="B62" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C62" s="46">
+      <c r="C62" s="49">
         <v>0</v>
       </c>
-      <c r="D62" s="46"/>
+      <c r="D62" s="49"/>
       <c r="K62" t="s">
         <v>98</v>
       </c>
@@ -39488,11 +39488,11 @@
       <c r="B63" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C63" s="46">
+      <c r="C63" s="49">
         <f>-SUMIFS(I$3:I$56,B$3:B$56,A$60,P$3:P$56,"xx",N$3:N$56,"x")</f>
         <v>0</v>
       </c>
-      <c r="D63" s="46"/>
+      <c r="D63" s="49"/>
       <c r="E63" s="2">
         <f>SUMIFS(Q$3:Q$56,B$3:B$56,A$60,P$3:P$56,"xx",N$3:N$56,"x")</f>
         <v>0</v>
@@ -39544,8 +39544,8 @@
       <c r="B65" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C65" s="48"/>
-      <c r="D65" s="48"/>
+      <c r="C65" s="45"/>
+      <c r="D65" s="45"/>
       <c r="I65">
         <v>33514</v>
       </c>
@@ -39564,8 +39564,8 @@
       <c r="B66" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C66" s="48"/>
-      <c r="D66" s="48"/>
+      <c r="C66" s="45"/>
+      <c r="D66" s="45"/>
       <c r="I66">
         <v>33379</v>
       </c>
@@ -39598,11 +39598,11 @@
       <c r="B68" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C68" s="45">
+      <c r="C68" s="46">
         <f>C64+C65+C66</f>
         <v>50515</v>
       </c>
-      <c r="D68" s="45"/>
+      <c r="D68" s="46"/>
       <c r="E68" s="1" t="s">
         <v>109</v>
       </c>
@@ -40842,11 +40842,11 @@
       <c r="B29" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C29" s="49">
+      <c r="C29" s="48">
         <f>SUMIFS(I$3:I$24,B$3:B$24,A$28,L$3:L$24,A$29)</f>
         <v>7205</v>
       </c>
-      <c r="D29" s="49"/>
+      <c r="D29" s="48"/>
       <c r="E29" s="3">
         <f>SUMIFS(Q$3:Q$24,B$3:B$24,A$28,L$3:L$24,A$29)</f>
         <v>22</v>
@@ -40881,10 +40881,10 @@
       <c r="B30" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C30" s="46">
+      <c r="C30" s="49">
         <v>0</v>
       </c>
-      <c r="D30" s="46"/>
+      <c r="D30" s="49"/>
       <c r="K30" t="s">
         <v>98</v>
       </c>
@@ -40908,11 +40908,11 @@
       <c r="B31" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C31" s="46">
+      <c r="C31" s="49">
         <f>-SUMIFS(I$3:I$24,B$3:B$24,A$28,P$3:P$24,"xx",N$3:N$24,"x")</f>
         <v>0</v>
       </c>
-      <c r="D31" s="46"/>
+      <c r="D31" s="49"/>
       <c r="E31" s="2">
         <f>SUMIFS(Q$3:Q$24,B$3:B$24,A$28,P$3:P$24,"xx",N$3:N$24,"x")</f>
         <v>0</v>
@@ -40964,8 +40964,8 @@
       <c r="B33" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C33" s="48"/>
-      <c r="D33" s="48"/>
+      <c r="C33" s="45"/>
+      <c r="D33" s="45"/>
       <c r="K33" s="2" t="s">
         <v>105</v>
       </c>
@@ -40981,8 +40981,8 @@
       <c r="B34" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C34" s="48"/>
-      <c r="D34" s="48"/>
+      <c r="C34" s="45"/>
+      <c r="D34" s="45"/>
       <c r="L34" s="9">
         <f>SUBTOTAL(9,L29:L33)</f>
         <v>2296</v>
@@ -40996,11 +40996,11 @@
       <c r="B36" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C36" s="45">
+      <c r="C36" s="46">
         <f>C32+C33+C34</f>
         <v>7205</v>
       </c>
-      <c r="D36" s="45"/>
+      <c r="D36" s="46"/>
       <c r="E36" s="1" t="s">
         <v>109</v>
       </c>
@@ -43920,11 +43920,11 @@
       <c r="B66" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C66" s="49">
+      <c r="C66" s="48">
         <f>SUMIFS(I$3:I$61,B$3:B$61,A$65,L$3:L$61,A$66)</f>
         <v>34740</v>
       </c>
-      <c r="D66" s="49"/>
+      <c r="D66" s="48"/>
       <c r="E66" s="3">
         <f>SUMIFS(Q$3:Q$61,B$3:B$61,A$65,L$3:L$61,A$66)</f>
         <v>59</v>
@@ -43959,10 +43959,10 @@
       <c r="B67" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C67" s="46">
+      <c r="C67" s="49">
         <v>0</v>
       </c>
-      <c r="D67" s="46"/>
+      <c r="D67" s="49"/>
       <c r="K67" t="s">
         <v>98</v>
       </c>
@@ -43986,11 +43986,11 @@
       <c r="B68" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C68" s="46">
+      <c r="C68" s="49">
         <f>-SUMIFS(I$3:I$61,B$3:B$61,A$65,P$3:P$61,"xx",N$3:N$61,"x")</f>
         <v>0</v>
       </c>
-      <c r="D68" s="46"/>
+      <c r="D68" s="49"/>
       <c r="E68" s="2">
         <f>SUMIFS(Q$3:Q$61,B$3:B$61,A$65,P$3:P$61,"xx",N$3:N$61,"x")</f>
         <v>0</v>
@@ -44034,8 +44034,8 @@
       <c r="B70" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C70" s="48"/>
-      <c r="D70" s="48"/>
+      <c r="C70" s="45"/>
+      <c r="D70" s="45"/>
       <c r="K70" s="2" t="s">
         <v>105</v>
       </c>
@@ -44051,8 +44051,8 @@
       <c r="B71" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C71" s="48"/>
-      <c r="D71" s="48"/>
+      <c r="C71" s="45"/>
+      <c r="D71" s="45"/>
       <c r="L71" s="9">
         <f>SUBTOTAL(9,L66:L70)</f>
         <v>26296</v>
@@ -44073,11 +44073,11 @@
       <c r="B73" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C73" s="45">
+      <c r="C73" s="46">
         <f>C69+C70+C71</f>
         <v>34740</v>
       </c>
-      <c r="D73" s="45"/>
+      <c r="D73" s="46"/>
       <c r="E73" s="1" t="s">
         <v>109</v>
       </c>
@@ -47295,11 +47295,11 @@
       <c r="B71" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C71" s="49">
+      <c r="C71" s="48">
         <f>SUMIFS(I$3:I$66,B$3:B$66,A$70,L$3:L$66,A$71)</f>
         <v>50540</v>
       </c>
-      <c r="D71" s="49"/>
+      <c r="D71" s="48"/>
       <c r="E71" s="3">
         <f>SUMIFS(Q$3:Q$66,B$3:B$66,A$70,L$3:L$66,A$71)</f>
         <v>64</v>
@@ -47333,10 +47333,10 @@
       <c r="B72" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C72" s="46">
+      <c r="C72" s="49">
         <v>0</v>
       </c>
-      <c r="D72" s="46"/>
+      <c r="D72" s="49"/>
       <c r="K72" t="s">
         <v>98</v>
       </c>
@@ -47359,11 +47359,11 @@
       <c r="B73" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C73" s="46">
+      <c r="C73" s="49">
         <f>-SUMIFS(I$3:I$66,B$3:B$66,A$70,P$3:P$66,"xx",N$3:N$66,"x")</f>
         <v>0</v>
       </c>
-      <c r="D73" s="46"/>
+      <c r="D73" s="49"/>
       <c r="E73" s="2">
         <f>SUMIFS(Q$3:Q$66,B$3:B$66,A$70,P$3:P$66,"xx",N$3:N$66,"x")</f>
         <v>0</v>
@@ -47413,8 +47413,8 @@
       <c r="B75" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C75" s="48"/>
-      <c r="D75" s="48"/>
+      <c r="C75" s="45"/>
+      <c r="D75" s="45"/>
       <c r="G75" s="10" t="s">
         <v>2580</v>
       </c>
@@ -47437,8 +47437,8 @@
       <c r="B76" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C76" s="48"/>
-      <c r="D76" s="48"/>
+      <c r="C76" s="45"/>
+      <c r="D76" s="45"/>
       <c r="L76" s="9">
         <f>SUBTOTAL(9,L71:L75)</f>
         <v>24613</v>
@@ -47452,11 +47452,11 @@
       <c r="B78" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C78" s="45">
+      <c r="C78" s="46">
         <f>C74+C75+C76</f>
         <v>50540</v>
       </c>
-      <c r="D78" s="45"/>
+      <c r="D78" s="46"/>
       <c r="E78" s="1" t="s">
         <v>109</v>
       </c>
@@ -50053,11 +50053,11 @@
       <c r="B58" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C58" s="49">
+      <c r="C58" s="48">
         <f>SUMIFS(I$3:I$53,B$3:B$53,A$57,L$3:L$53,A$58)</f>
         <v>33955</v>
       </c>
-      <c r="D58" s="49"/>
+      <c r="D58" s="48"/>
       <c r="E58" s="3">
         <f>SUMIFS(Q$3:Q$53,B$3:B$53,A$57,L$3:L$53,A$58)</f>
         <v>50</v>
@@ -50092,10 +50092,10 @@
       <c r="B59" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C59" s="46">
+      <c r="C59" s="49">
         <v>0</v>
       </c>
-      <c r="D59" s="46"/>
+      <c r="D59" s="49"/>
       <c r="K59" t="s">
         <v>98</v>
       </c>
@@ -50119,11 +50119,11 @@
       <c r="B60" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C60" s="46">
+      <c r="C60" s="49">
         <f>-SUMIFS(I$3:I$53,B$3:B$53,A$57,P$3:P$53,"xx",N$3:N$53,"x")</f>
         <v>-765</v>
       </c>
-      <c r="D60" s="46"/>
+      <c r="D60" s="49"/>
       <c r="E60" s="2">
         <f>SUMIFS(Q$3:Q$53,B$3:B$53,A$57,P$3:P$53,"xx",N$3:N$53,"x")</f>
         <v>1</v>
@@ -50169,8 +50169,8 @@
       <c r="B62" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C62" s="48"/>
-      <c r="D62" s="48"/>
+      <c r="C62" s="45"/>
+      <c r="D62" s="45"/>
       <c r="K62" s="2" t="s">
         <v>105</v>
       </c>
@@ -50186,8 +50186,8 @@
       <c r="B63" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C63" s="48"/>
-      <c r="D63" s="48"/>
+      <c r="C63" s="45"/>
+      <c r="D63" s="45"/>
       <c r="L63" s="9">
         <f>SUBTOTAL(9,L58:L62)</f>
         <v>19225</v>
@@ -50201,11 +50201,11 @@
       <c r="B65" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C65" s="45">
+      <c r="C65" s="46">
         <f>C61+C62+C63</f>
         <v>33190</v>
       </c>
-      <c r="D65" s="45"/>
+      <c r="D65" s="46"/>
       <c r="E65" s="1" t="s">
         <v>109</v>
       </c>
@@ -56061,11 +56061,11 @@
       <c r="B130" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C130" s="49">
+      <c r="C130" s="48">
         <f>SUMIFS(I$3:I$125,B$3:B$125,A$129,L$3:L$125,A$130)</f>
         <v>88515</v>
       </c>
-      <c r="D130" s="49"/>
+      <c r="D130" s="48"/>
       <c r="E130" s="3">
         <f>SUMIFS(Q$3:Q$125,B$3:B$125,A$129,L$3:L$125,A$130)</f>
         <v>120</v>
@@ -56100,10 +56100,10 @@
       <c r="B131" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C131" s="46">
+      <c r="C131" s="49">
         <v>0</v>
       </c>
-      <c r="D131" s="46"/>
+      <c r="D131" s="49"/>
       <c r="K131" t="s">
         <v>98</v>
       </c>
@@ -56127,11 +56127,11 @@
       <c r="B132" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C132" s="46">
+      <c r="C132" s="49">
         <f>-SUMIFS(I$3:I$125,B$3:B$125,A$129,P$3:P$125,"xx",N$3:N$125,"x")</f>
         <v>-5870</v>
       </c>
-      <c r="D132" s="46"/>
+      <c r="D132" s="49"/>
       <c r="E132" s="2">
         <f>SUMIFS(Q$3:Q$125,B$3:B$125,A$129,P$3:P$125,"xx",N$3:N$125,"x")</f>
         <v>7</v>
@@ -56175,8 +56175,8 @@
       <c r="B134" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C134" s="48"/>
-      <c r="D134" s="48"/>
+      <c r="C134" s="45"/>
+      <c r="D134" s="45"/>
       <c r="K134" s="2" t="s">
         <v>105</v>
       </c>
@@ -56192,10 +56192,10 @@
       <c r="B135" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C135" s="48">
+      <c r="C135" s="45">
         <v>790</v>
       </c>
-      <c r="D135" s="48"/>
+      <c r="D135" s="45"/>
       <c r="L135" s="9">
         <f>SUBTOTAL(9,L130:L134)</f>
         <v>24905</v>
@@ -56222,11 +56222,11 @@
       <c r="B137" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C137" s="45">
+      <c r="C137" s="46">
         <f>C133+C134+C135</f>
         <v>83435</v>
       </c>
-      <c r="D137" s="45"/>
+      <c r="D137" s="46"/>
       <c r="E137" s="1" t="s">
         <v>109</v>
       </c>
@@ -58698,11 +58698,11 @@
       <c r="B54" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C54" s="49">
+      <c r="C54" s="48">
         <f>SUMIFS(I$3:I$49,B$3:B$49,A$53,L$3:L$49,A$54)</f>
         <v>38441</v>
       </c>
-      <c r="D54" s="49"/>
+      <c r="D54" s="48"/>
       <c r="E54" s="3">
         <f>SUMIFS(Q$3:Q$49,B$3:B$49,A$53,L$3:L$49,A$54)</f>
         <v>45</v>
@@ -58737,10 +58737,10 @@
       <c r="B55" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C55" s="46" t="s">
+      <c r="C55" s="49" t="s">
         <v>3251</v>
       </c>
-      <c r="D55" s="46"/>
+      <c r="D55" s="49"/>
       <c r="K55" t="s">
         <v>98</v>
       </c>
@@ -58764,11 +58764,11 @@
       <c r="B56" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C56" s="46">
+      <c r="C56" s="49">
         <f>-SUMIFS(I$3:I$49,B$3:B$49,A$53,P$3:P$49,"xx",N$3:N$49,"x")</f>
         <v>-750</v>
       </c>
-      <c r="D56" s="46"/>
+      <c r="D56" s="49"/>
       <c r="E56" s="2">
         <f>SUMIFS(Q$3:Q$49,B$3:B$49,A$53,P$3:P$49,"xx",N$3:N$49,"x")</f>
         <v>1</v>
@@ -58820,8 +58820,8 @@
       <c r="B58" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C58" s="48"/>
-      <c r="D58" s="48"/>
+      <c r="C58" s="45"/>
+      <c r="D58" s="45"/>
       <c r="K58" s="2" t="s">
         <v>105</v>
       </c>
@@ -58843,8 +58843,8 @@
       <c r="B59" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C59" s="48"/>
-      <c r="D59" s="48"/>
+      <c r="C59" s="45"/>
+      <c r="D59" s="45"/>
       <c r="L59" s="9">
         <f>SUBTOTAL(9,L54:L58)</f>
         <v>18525</v>
@@ -58865,11 +58865,11 @@
       <c r="B61" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C61" s="45">
+      <c r="C61" s="46">
         <f>C57+C58+C59</f>
         <v>37691</v>
       </c>
-      <c r="D61" s="45"/>
+      <c r="D61" s="46"/>
       <c r="E61" s="1" t="s">
         <v>109</v>
       </c>
@@ -58926,11 +58926,11 @@
       <c r="B64" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C64" s="49">
+      <c r="C64" s="48">
         <f>SUMIFS(I$3:I$49,B$3:B$49,A$63,L$3:L$49,A$64)</f>
         <v>450</v>
       </c>
-      <c r="D64" s="49"/>
+      <c r="D64" s="48"/>
       <c r="E64" s="3">
         <f>SUMIFS(Q$3:Q$49,B$3:B$49,A$63,L$3:L$49,A$64)</f>
         <v>1</v>
@@ -58946,10 +58946,10 @@
       <c r="B65" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C65" s="46">
+      <c r="C65" s="49">
         <v>0</v>
       </c>
-      <c r="D65" s="46"/>
+      <c r="D65" s="49"/>
       <c r="K65" s="2" t="s">
         <v>102</v>
       </c>
@@ -58958,8 +58958,8 @@
       <c r="B66" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C66" s="46"/>
-      <c r="D66" s="46"/>
+      <c r="C66" s="49"/>
+      <c r="D66" s="49"/>
       <c r="E66" s="2"/>
       <c r="K66" s="2" t="s">
         <v>105</v>
@@ -58992,8 +58992,8 @@
       <c r="B68" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C68" s="48"/>
-      <c r="D68" s="48"/>
+      <c r="C68" s="45"/>
+      <c r="D68" s="45"/>
       <c r="L68" s="9">
         <f>SUBTOTAL(9,L62:L66)</f>
         <v>10016</v>
@@ -59007,8 +59007,8 @@
       <c r="B69" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C69" s="48"/>
-      <c r="D69" s="48"/>
+      <c r="C69" s="45"/>
+      <c r="D69" s="45"/>
     </row>
     <row r="70" spans="2:13" x14ac:dyDescent="0.25">
       <c r="K70" s="7" t="s">
@@ -59025,11 +59025,11 @@
       <c r="B71" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C71" s="45">
+      <c r="C71" s="46">
         <f>C67+C68+C69</f>
         <v>450</v>
       </c>
-      <c r="D71" s="45"/>
+      <c r="D71" s="46"/>
       <c r="E71" s="1" t="s">
         <v>109</v>
       </c>
@@ -59152,22 +59152,22 @@
     </sortState>
   </autoFilter>
   <mergeCells count="16">
-    <mergeCell ref="C53:D53"/>
-    <mergeCell ref="C54:D54"/>
-    <mergeCell ref="C55:D55"/>
-    <mergeCell ref="C56:D56"/>
-    <mergeCell ref="C57:D57"/>
-    <mergeCell ref="C58:D58"/>
-    <mergeCell ref="C59:D59"/>
-    <mergeCell ref="C61:D61"/>
-    <mergeCell ref="C63:D63"/>
-    <mergeCell ref="C64:D64"/>
     <mergeCell ref="C71:D71"/>
     <mergeCell ref="C65:D65"/>
     <mergeCell ref="C66:D66"/>
     <mergeCell ref="C67:D67"/>
     <mergeCell ref="C68:D68"/>
     <mergeCell ref="C69:D69"/>
+    <mergeCell ref="C58:D58"/>
+    <mergeCell ref="C59:D59"/>
+    <mergeCell ref="C61:D61"/>
+    <mergeCell ref="C63:D63"/>
+    <mergeCell ref="C64:D64"/>
+    <mergeCell ref="C53:D53"/>
+    <mergeCell ref="C54:D54"/>
+    <mergeCell ref="C55:D55"/>
+    <mergeCell ref="C56:D56"/>
+    <mergeCell ref="C57:D57"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
 </worksheet>
@@ -61966,11 +61966,11 @@
       <c r="B65" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C65" s="49">
+      <c r="C65" s="48">
         <f>SUMIFS(I$3:I$60,B$3:B$60,A$64,L$3:L$60,A$65)</f>
         <v>46230</v>
       </c>
-      <c r="D65" s="49"/>
+      <c r="D65" s="48"/>
       <c r="E65" s="3">
         <f>SUMIFS(Q$3:Q$60,B$3:B$60,A$64,L$3:L$60,A$65)</f>
         <v>58</v>
@@ -62005,10 +62005,10 @@
       <c r="B66" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C66" s="46">
+      <c r="C66" s="49">
         <v>0</v>
       </c>
-      <c r="D66" s="46"/>
+      <c r="D66" s="49"/>
       <c r="K66" t="s">
         <v>98</v>
       </c>
@@ -62032,11 +62032,11 @@
       <c r="B67" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C67" s="46">
+      <c r="C67" s="49">
         <f>-SUMIFS(I$3:I$60,B$3:B$60,A$64,P$3:P$60,"xx",N$3:N$60,"x")</f>
         <v>0</v>
       </c>
-      <c r="D67" s="46"/>
+      <c r="D67" s="49"/>
       <c r="E67" s="2">
         <f>SUMIFS(Q$3:Q$60,B$3:B$60,A$64,P$3:P$60,"xx",N$3:N$60,"x")</f>
         <v>0</v>
@@ -62080,8 +62080,8 @@
       <c r="B69" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C69" s="48"/>
-      <c r="D69" s="48"/>
+      <c r="C69" s="45"/>
+      <c r="D69" s="45"/>
       <c r="K69" s="2" t="s">
         <v>105</v>
       </c>
@@ -62097,8 +62097,8 @@
       <c r="B70" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C70" s="48"/>
-      <c r="D70" s="48"/>
+      <c r="C70" s="45"/>
+      <c r="D70" s="45"/>
       <c r="L70" s="9">
         <f>SUBTOTAL(9,L65:L69)</f>
         <v>18610</v>
@@ -62119,11 +62119,11 @@
       <c r="B72" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C72" s="45">
+      <c r="C72" s="46">
         <f>C68+C69+C70</f>
         <v>46230</v>
       </c>
-      <c r="D72" s="45"/>
+      <c r="D72" s="46"/>
       <c r="E72" s="1" t="s">
         <v>109</v>
       </c>
@@ -65135,11 +65135,11 @@
       <c r="B58" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C58" s="49">
+      <c r="C58" s="48">
         <f>SUMIFS(I$3:I$53,B$3:B$53,A$57,L$3:L$53,A$58)</f>
         <v>29790</v>
       </c>
-      <c r="D58" s="49"/>
+      <c r="D58" s="48"/>
       <c r="E58" s="3">
         <f>SUMIFS(Q$3:Q$53,B$3:B$53,A$57,L$3:L$53,A$58)</f>
         <v>51</v>
@@ -65174,10 +65174,10 @@
       <c r="B59" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C59" s="46">
+      <c r="C59" s="49">
         <v>0</v>
       </c>
-      <c r="D59" s="46"/>
+      <c r="D59" s="49"/>
       <c r="K59" t="s">
         <v>98</v>
       </c>
@@ -65201,11 +65201,11 @@
       <c r="B60" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C60" s="46">
+      <c r="C60" s="49">
         <f>-SUMIFS(I$3:I$53,B$3:B$53,A$57,P$3:P$53,"xx",N$3:N$53,"x")</f>
         <v>0</v>
       </c>
-      <c r="D60" s="46"/>
+      <c r="D60" s="49"/>
       <c r="E60" s="2">
         <f>SUMIFS(Q$3:Q$53,B$3:B$53,A$57,P$3:P$53,"xx",N$3:N$53,"x")</f>
         <v>0</v>
@@ -65257,8 +65257,8 @@
       <c r="B62" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C62" s="48"/>
-      <c r="D62" s="48"/>
+      <c r="C62" s="45"/>
+      <c r="D62" s="45"/>
       <c r="K62" s="2" t="s">
         <v>105</v>
       </c>
@@ -65274,8 +65274,8 @@
       <c r="B63" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C63" s="48"/>
-      <c r="D63" s="48"/>
+      <c r="C63" s="45"/>
+      <c r="D63" s="45"/>
       <c r="K63" s="10" t="s">
         <v>323</v>
       </c>
@@ -65297,11 +65297,11 @@
       <c r="B65" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C65" s="45">
+      <c r="C65" s="46">
         <f>C61+C62+C63</f>
         <v>29790</v>
       </c>
-      <c r="D65" s="45"/>
+      <c r="D65" s="46"/>
       <c r="E65" s="1" t="s">
         <v>109</v>
       </c>
@@ -67286,11 +67286,11 @@
       <c r="B49" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C49" s="49">
+      <c r="C49" s="48">
         <f>SUMIFS(I$3:I$44,B$3:B$44,A$48,L$3:L$44,A$49)</f>
         <v>20745</v>
       </c>
-      <c r="D49" s="49"/>
+      <c r="D49" s="48"/>
       <c r="E49" s="3">
         <f>SUMIFS(Q$3:Q$44,B$3:B$44,A$48,L$3:L$44,A$49)</f>
         <v>40</v>
@@ -67325,10 +67325,10 @@
       <c r="B50" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C50" s="46">
+      <c r="C50" s="49">
         <v>0</v>
       </c>
-      <c r="D50" s="46"/>
+      <c r="D50" s="49"/>
       <c r="K50" t="s">
         <v>98</v>
       </c>
@@ -67352,11 +67352,11 @@
       <c r="B51" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C51" s="46">
+      <c r="C51" s="49">
         <f>-SUMIFS(I$3:I$44,B$3:B$44,A$48,P$3:P$44,"xx",N$3:N$44,"x")</f>
         <v>-970</v>
       </c>
-      <c r="D51" s="46"/>
+      <c r="D51" s="49"/>
       <c r="E51" s="2">
         <f>SUMIFS(Q$3:Q$44,B$3:B$44,A$48,P$3:P$44,"xx",N$3:N$44,"x")</f>
         <v>2</v>
@@ -67406,8 +67406,8 @@
       <c r="B53" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C53" s="48"/>
-      <c r="D53" s="48"/>
+      <c r="C53" s="45"/>
+      <c r="D53" s="45"/>
       <c r="K53" s="2" t="s">
         <v>105</v>
       </c>
@@ -67423,8 +67423,8 @@
       <c r="B54" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C54" s="48"/>
-      <c r="D54" s="48"/>
+      <c r="C54" s="45"/>
+      <c r="D54" s="45"/>
       <c r="L54" s="9">
         <f>SUBTOTAL(9,L49:L53)</f>
         <v>8722</v>
@@ -67445,11 +67445,11 @@
       <c r="B56" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C56" s="45">
+      <c r="C56" s="46">
         <f>C52+C53+C54</f>
         <v>19775</v>
       </c>
-      <c r="D56" s="45"/>
+      <c r="D56" s="46"/>
       <c r="E56" s="1" t="s">
         <v>109</v>
       </c>
@@ -69929,11 +69929,11 @@
       <c r="B60" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C60" s="49">
+      <c r="C60" s="48">
         <f>SUMIFS(I$3:I$55,B$3:B$55,A$59,L$3:L$55,A$60)</f>
         <v>33510</v>
       </c>
-      <c r="D60" s="49"/>
+      <c r="D60" s="48"/>
       <c r="E60" s="3">
         <f>SUMIFS(Q$3:Q$55,B$3:B$55,A$59,L$3:L$55,A$60)</f>
         <v>52</v>
@@ -69968,10 +69968,10 @@
       <c r="B61" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C61" s="46">
+      <c r="C61" s="49">
         <v>0</v>
       </c>
-      <c r="D61" s="46"/>
+      <c r="D61" s="49"/>
       <c r="K61" t="s">
         <v>98</v>
       </c>
@@ -69995,11 +69995,11 @@
       <c r="B62" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C62" s="46">
+      <c r="C62" s="49">
         <f>-SUMIFS(I$3:I$55,B$3:B$55,A$59,P$3:P$55,"xx",N$3:N$55,"x")</f>
         <v>-860</v>
       </c>
-      <c r="D62" s="46"/>
+      <c r="D62" s="49"/>
       <c r="E62" s="2">
         <f>SUMIFS(Q$3:Q$55,B$3:B$55,A$59,P$3:P$55,"xx",N$3:N$55,"x")</f>
         <v>1</v>
@@ -70051,8 +70051,8 @@
       <c r="B64" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C64" s="48"/>
-      <c r="D64" s="48"/>
+      <c r="C64" s="45"/>
+      <c r="D64" s="45"/>
       <c r="K64" s="2" t="s">
         <v>105</v>
       </c>
@@ -70068,8 +70068,8 @@
       <c r="B65" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C65" s="48"/>
-      <c r="D65" s="48"/>
+      <c r="C65" s="45"/>
+      <c r="D65" s="45"/>
       <c r="L65" s="9">
         <f>SUBTOTAL(9,L60:L64)</f>
         <v>8748</v>
@@ -70083,11 +70083,11 @@
       <c r="B67" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C67" s="45">
+      <c r="C67" s="46">
         <f>C63+C64+C65</f>
         <v>32650</v>
       </c>
-      <c r="D67" s="45"/>
+      <c r="D67" s="46"/>
       <c r="E67" s="1" t="s">
         <v>109</v>
       </c>
@@ -71484,7 +71484,7 @@
         <f>SUMIFS(I$3:I$29,B$3:B$29,A$33,L$3:L$29,A$34)+I32</f>
         <v>24145</v>
       </c>
-      <c r="D34" s="49"/>
+      <c r="D34" s="48"/>
       <c r="E34" s="3">
         <f>SUMIFS(Q$3:Q$29,B$3:B$29,A$33,L$3:L$29,A$34)</f>
         <v>25</v>
@@ -71519,10 +71519,10 @@
       <c r="B35" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C35" s="46">
+      <c r="C35" s="49">
         <v>0</v>
       </c>
-      <c r="D35" s="46"/>
+      <c r="D35" s="49"/>
       <c r="K35" t="s">
         <v>98</v>
       </c>
@@ -71546,11 +71546,11 @@
       <c r="B36" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C36" s="46">
+      <c r="C36" s="49">
         <f>-SUMIFS(I$3:I$29,B$3:B$29,A$33,P$3:P$29,"xx",N$3:N$29,"x")</f>
         <v>-1715</v>
       </c>
-      <c r="D36" s="46"/>
+      <c r="D36" s="49"/>
       <c r="E36" s="2">
         <f>SUMIFS(Q$3:Q$29,B$3:B$29,A$33,P$3:P$29,"xx",N$3:N$29,"x")</f>
         <v>2</v>
@@ -71601,10 +71601,10 @@
       <c r="B38" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C38" s="48">
+      <c r="C38" s="45">
         <v>-70</v>
       </c>
-      <c r="D38" s="48"/>
+      <c r="D38" s="45"/>
       <c r="K38" s="2" t="s">
         <v>105</v>
       </c>
@@ -71623,8 +71623,8 @@
       <c r="B39" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C39" s="48"/>
-      <c r="D39" s="48"/>
+      <c r="C39" s="45"/>
+      <c r="D39" s="45"/>
       <c r="K39" s="10" t="s">
         <v>664</v>
       </c>
@@ -71661,11 +71661,11 @@
       <c r="B42" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C42" s="45">
+      <c r="C42" s="46">
         <f>C37+C38+C39</f>
         <v>22360</v>
       </c>
-      <c r="D42" s="45"/>
+      <c r="D42" s="46"/>
       <c r="E42" s="1" t="s">
         <v>109</v>
       </c>
@@ -73995,11 +73995,11 @@
       <c r="B52" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C52" s="49">
+      <c r="C52" s="48">
         <f>SUMIFS(I$3:I$47,B$3:B$47,A$51,L$3:L$47,A$52)</f>
         <v>25380</v>
       </c>
-      <c r="D52" s="49"/>
+      <c r="D52" s="48"/>
       <c r="E52" s="3">
         <f>SUMIFS(Q$3:Q$47,B$3:B$47,A$51,L$3:L$47,A$52)</f>
         <v>43</v>
@@ -74034,10 +74034,10 @@
       <c r="B53" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C53" s="46">
+      <c r="C53" s="49">
         <v>0</v>
       </c>
-      <c r="D53" s="46"/>
+      <c r="D53" s="49"/>
       <c r="K53" t="s">
         <v>98</v>
       </c>
@@ -74061,11 +74061,11 @@
       <c r="B54" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C54" s="46">
+      <c r="C54" s="49">
         <f>-SUMIFS(I$3:I$47,B$3:B$47,A$51,P$3:P$47,"xx",N$3:N$47,"x")</f>
         <v>-710</v>
       </c>
-      <c r="D54" s="46"/>
+      <c r="D54" s="49"/>
       <c r="E54" s="2">
         <f>SUMIFS(Q$3:Q$47,B$3:B$47,A$51,P$3:P$47,"xx",N$3:N$47,"x")</f>
         <v>3</v>
@@ -74117,8 +74117,8 @@
       <c r="B56" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C56" s="48"/>
-      <c r="D56" s="48"/>
+      <c r="C56" s="45"/>
+      <c r="D56" s="45"/>
       <c r="K56" s="2" t="s">
         <v>105</v>
       </c>
@@ -74134,8 +74134,8 @@
       <c r="B57" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C57" s="48"/>
-      <c r="D57" s="48"/>
+      <c r="C57" s="45"/>
+      <c r="D57" s="45"/>
       <c r="L57" s="9">
         <f>SUBTOTAL(9,L52:L56)</f>
         <v>4847</v>
@@ -74156,11 +74156,11 @@
       <c r="B59" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C59" s="45">
+      <c r="C59" s="46">
         <f>C55+C56+C57</f>
         <v>24670</v>
       </c>
-      <c r="D59" s="45"/>
+      <c r="D59" s="46"/>
       <c r="E59" s="1" t="s">
         <v>109</v>
       </c>
@@ -76175,11 +76175,11 @@
       <c r="B44" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C44" s="49">
+      <c r="C44" s="48">
         <f>SUMIFS(I$3:I$39,B$3:B$39,A$43,L$3:L$39,A$44)</f>
         <v>23985</v>
       </c>
-      <c r="D44" s="49"/>
+      <c r="D44" s="48"/>
       <c r="E44" s="3">
         <f>SUMIFS(Q$3:Q$39,B$3:B$39,A$43,L$3:L$39,A$44)</f>
         <v>37</v>
@@ -76210,10 +76210,10 @@
       <c r="B45" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C45" s="46">
+      <c r="C45" s="49">
         <v>0</v>
       </c>
-      <c r="D45" s="46"/>
+      <c r="D45" s="49"/>
       <c r="K45" t="s">
         <v>98</v>
       </c>
@@ -76237,11 +76237,11 @@
       <c r="B46" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C46" s="46">
+      <c r="C46" s="49">
         <f>-SUMIFS(I$3:I$39,B$3:B$39,A$43,P$3:P$39,"xx",N$3:N$39,"x")</f>
         <v>0</v>
       </c>
-      <c r="D46" s="46"/>
+      <c r="D46" s="49"/>
       <c r="E46" s="2">
         <f>SUMIFS(Q$3:Q$39,B$3:B$39,A$43,P$3:P$39,"xx",N$3:N$39,"x")</f>
         <v>0</v>
@@ -76293,8 +76293,8 @@
       <c r="B48" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C48" s="48"/>
-      <c r="D48" s="48"/>
+      <c r="C48" s="45"/>
+      <c r="D48" s="45"/>
       <c r="K48" s="2" t="s">
         <v>105</v>
       </c>
@@ -76310,8 +76310,8 @@
       <c r="B49" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C49" s="48"/>
-      <c r="D49" s="48"/>
+      <c r="C49" s="45"/>
+      <c r="D49" s="45"/>
       <c r="L49" s="9">
         <f>SUBTOTAL(9,L44:L48)</f>
         <v>7556</v>
@@ -76325,11 +76325,11 @@
       <c r="B51" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C51" s="45">
+      <c r="C51" s="46">
         <f>C47+C48+C49</f>
         <v>23985</v>
       </c>
-      <c r="D51" s="45"/>
+      <c r="D51" s="46"/>
       <c r="E51" s="1" t="s">
         <v>109</v>
       </c>
@@ -79005,11 +79005,11 @@
       <c r="B59" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="C59" s="49">
+      <c r="C59" s="48">
         <f>SUMIFS(I$3:I$55,B$3:B$55,A$58,L$3:L$55,A$59)</f>
         <v>43676</v>
       </c>
-      <c r="D59" s="49"/>
+      <c r="D59" s="48"/>
       <c r="E59" s="3">
         <f>SUMIFS(Q$3:Q$55,B$3:B$55,A$58,L$3:L$55,A$59)</f>
         <v>51</v>
@@ -79040,10 +79040,10 @@
       <c r="B60" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="C60" s="46">
+      <c r="C60" s="49">
         <v>0</v>
       </c>
-      <c r="D60" s="46"/>
+      <c r="D60" s="49"/>
       <c r="K60" t="s">
         <v>98</v>
       </c>
@@ -79067,11 +79067,11 @@
       <c r="B61" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="C61" s="46">
+      <c r="C61" s="49">
         <f>-SUMIFS(I$3:I$55,B$3:B$55,A$58,P$3:P$55,"xx",N$3:N$55,"x")</f>
         <v>-975</v>
       </c>
-      <c r="D61" s="46"/>
+      <c r="D61" s="49"/>
       <c r="E61" s="2">
         <f>SUMIFS(Q$3:Q$55,B$3:B$55,A$58,P$3:P$55,"xx",N$3:N$55,"x")</f>
         <v>2</v>
@@ -79121,8 +79121,8 @@
       <c r="B63" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="C63" s="48"/>
-      <c r="D63" s="48"/>
+      <c r="C63" s="45"/>
+      <c r="D63" s="45"/>
       <c r="K63" s="2" t="s">
         <v>105</v>
       </c>
@@ -79138,8 +79138,8 @@
       <c r="B64" s="8" t="s">
         <v>107</v>
       </c>
-      <c r="C64" s="48"/>
-      <c r="D64" s="48"/>
+      <c r="C64" s="45"/>
+      <c r="D64" s="45"/>
       <c r="L64" s="9">
         <f>SUBTOTAL(9,L59:L63)</f>
         <v>9811</v>
@@ -79153,11 +79153,11 @@
       <c r="B66" s="1" t="s">
         <v>108</v>
       </c>
-      <c r="C66" s="45">
+      <c r="C66" s="46">
         <f>C62+C63+C64</f>
         <v>42701</v>
       </c>
-      <c r="D66" s="45"/>
+      <c r="D66" s="46"/>
       <c r="E66" s="1" t="s">
         <v>109</v>
       </c>

</xml_diff>